<commit_message>
Commit de L création de comparaisons
</commit_message>
<xml_diff>
--- a/data/raw/PM/PM_Montrouge.xlsx
+++ b/data/raw/PM/PM_Montrouge.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1795,40 +1795,40 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Mairie - Montrouge</t>
+          <t>Association mosquée de Montrouge</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>mairie</t>
+          <t>lieu de culte</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>api-lannuaire.service-public.fr + geocodage BAN</t>
+          <t>OpenStreetMap</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>48.818819</v>
+        <v>48.8125835</v>
       </c>
       <c r="E50" t="n">
-        <v>2.319869</v>
+        <v>2.3131517</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>48.818819, 2.319869</t>
+          <t>48.8125835, 2.3131517</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>La Poste Montrouge-Vache Noire</t>
+          <t>Centre évangélique international Évidence</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>poste</t>
+          <t>lieu de culte</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1837,26 +1837,26 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>48.8123121</v>
+        <v>48.8145108</v>
       </c>
       <c r="E51" t="n">
-        <v>2.3257731</v>
+        <v>2.3172515</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>48.8123121, 2.3257731</t>
+          <t>48.8145108, 2.3172515</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>La poste Montrouge Verdier</t>
+          <t>Oratoire Bienheureux Charles de Foucauld</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>poste</t>
+          <t>lieu de culte</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1865,26 +1865,26 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>48.8151689</v>
+        <v>48.8147869</v>
       </c>
       <c r="E52" t="n">
-        <v>2.3185804</v>
+        <v>2.3188595</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>48.8151689, 2.3185804</t>
+          <t>48.8147869, 2.3188595</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Mail Boxes Etc</t>
+          <t>lieu de culte sans nom</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>poste</t>
+          <t>lieu de culte</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1893,26 +1893,26 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>48.8160054</v>
+        <v>48.8180645</v>
       </c>
       <c r="E53" t="n">
-        <v>2.3210609</v>
+        <v>2.3185015</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>48.8160054, 2.3210609</t>
+          <t>48.8180645, 2.3185015</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Parcel Centre Vinted Go</t>
+          <t>Église Protestante Unie</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>poste</t>
+          <t>lieu de culte</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1921,26 +1921,26 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>48.8132586</v>
+        <v>48.8176105</v>
       </c>
       <c r="E54" t="n">
-        <v>2.3283416</v>
+        <v>2.3117168</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>48.8132586, 2.3283416</t>
+          <t>48.8176105, 2.3117168</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Relais Poste</t>
+          <t>Église Saint-Jacques-le-Majeur</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>poste</t>
+          <t>lieu de culte</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1949,14 +1949,406 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>48.8138579</v>
+        <v>48.8181396</v>
       </c>
       <c r="E55" t="n">
-        <v>2.3075651</v>
+        <v>2.3204543</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>48.8138579, 2.3075651</t>
+          <t>48.8181396, 2.3204543</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Église Saint-Joseph-Saint-Raymond</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>lieu de culte</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>48.8145944</v>
+      </c>
+      <c r="E56" t="n">
+        <v>2.3095679</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>48.8145944, 2.3095679</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Église Saint-Luc</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>lieu de culte</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>48.8108006</v>
+      </c>
+      <c r="E57" t="n">
+        <v>2.3234878</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>48.8108006, 2.3234878</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Église Évangelique de Salem</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>lieu de culte</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>48.810885</v>
+      </c>
+      <c r="E58" t="n">
+        <v>2.3079518</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>48.810885, 2.3079518</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Mairie - Montrouge</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>mairie</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>api-lannuaire.service-public.fr + geocodage BAN</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>48.818819</v>
+      </c>
+      <c r="E59" t="n">
+        <v>2.319869</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>48.818819, 2.319869</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Pharmacie Renard</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>pharmacie</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>48.8160855</v>
+      </c>
+      <c r="E60" t="n">
+        <v>2.3085881</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>48.8160855, 2.3085881</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Pharmacie Tuffier</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>pharmacie</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>48.8112481</v>
+      </c>
+      <c r="E61" t="n">
+        <v>2.3145403</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>48.8112481, 2.3145403</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Pharmacie de Paris</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>pharmacie</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>48.8185287</v>
+      </c>
+      <c r="E62" t="n">
+        <v>2.3225912</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>48.8185287, 2.3225912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Pharmacie de l'Aquapol</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>pharmacie</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>48.814625</v>
+      </c>
+      <c r="E63" t="n">
+        <v>2.32043</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>48.814625, 2.32043</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Pharmacie de l'Église</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>pharmacie</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>48.8178715</v>
+      </c>
+      <c r="E64" t="n">
+        <v>2.3190587</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>48.8178715, 2.3190587</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Pharmacie du Fort</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>pharmacie</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>48.8119254</v>
+      </c>
+      <c r="E65" t="n">
+        <v>2.3233672</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>48.8119254, 2.3233672</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Pharmacie du Marché</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>pharmacie</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>48.8166678</v>
+      </c>
+      <c r="E66" t="n">
+        <v>2.3212215</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>48.8166678, 2.3212215</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Pharmacie du Parc</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>pharmacie</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>48.8133473</v>
+      </c>
+      <c r="E67" t="n">
+        <v>2.3162607</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>48.8133473, 2.3162607</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Pharmacie du Square</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>pharmacie</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>48.8135808</v>
+      </c>
+      <c r="E68" t="n">
+        <v>2.3070756</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>48.8135808, 2.3070756</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>pharmacieCOS</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>pharmacie</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>48.8163976</v>
+      </c>
+      <c r="E69" t="n">
+        <v>2.3113604</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>48.8163976, 2.3113604</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
pb d'enregistrement pour la comparaison
</commit_message>
<xml_diff>
--- a/data/raw/PM/PM_Montrouge.xlsx
+++ b/data/raw/PM/PM_Montrouge.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,36 +425,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nom</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>latitude</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>longitude</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>coordonnees</t>
         </is>
@@ -1767,588 +1779,28 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Police municipale</t>
+          <t>Mairie - Montrouge</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>gendarmerie</t>
+          <t>mairie</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>OpenStreetMap</t>
+          <t>api-lannuaire.service-public.fr + geocodage BAN</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>48.8156606</v>
+        <v>48.818819</v>
       </c>
       <c r="E49" t="n">
-        <v>2.3195764</v>
+        <v>2.319869</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>48.8156606, 2.3195764</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Association mosquée de Montrouge</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>lieu de culte</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D50" t="n">
-        <v>48.8125835</v>
-      </c>
-      <c r="E50" t="n">
-        <v>2.3131517</v>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>48.8125835, 2.3131517</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Centre évangélique international Évidence</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>lieu de culte</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D51" t="n">
-        <v>48.8145108</v>
-      </c>
-      <c r="E51" t="n">
-        <v>2.3172515</v>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>48.8145108, 2.3172515</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Oratoire Bienheureux Charles de Foucauld</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>lieu de culte</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D52" t="n">
-        <v>48.8147869</v>
-      </c>
-      <c r="E52" t="n">
-        <v>2.3188595</v>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>48.8147869, 2.3188595</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>lieu de culte sans nom</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>lieu de culte</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
-        <v>48.8180645</v>
-      </c>
-      <c r="E53" t="n">
-        <v>2.3185015</v>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>48.8180645, 2.3185015</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Église Protestante Unie</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>lieu de culte</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D54" t="n">
-        <v>48.8176105</v>
-      </c>
-      <c r="E54" t="n">
-        <v>2.3117168</v>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>48.8176105, 2.3117168</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Église Saint-Jacques-le-Majeur</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>lieu de culte</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D55" t="n">
-        <v>48.8181396</v>
-      </c>
-      <c r="E55" t="n">
-        <v>2.3204543</v>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>48.8181396, 2.3204543</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Église Saint-Joseph-Saint-Raymond</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>lieu de culte</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D56" t="n">
-        <v>48.8145944</v>
-      </c>
-      <c r="E56" t="n">
-        <v>2.3095679</v>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>48.8145944, 2.3095679</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Église Saint-Luc</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>lieu de culte</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D57" t="n">
-        <v>48.8108006</v>
-      </c>
-      <c r="E57" t="n">
-        <v>2.3234878</v>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>48.8108006, 2.3234878</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Église Évangelique de Salem</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>lieu de culte</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D58" t="n">
-        <v>48.810885</v>
-      </c>
-      <c r="E58" t="n">
-        <v>2.3079518</v>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>48.810885, 2.3079518</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Mairie - Montrouge</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>mairie</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>api-lannuaire.service-public.fr + geocodage BAN</t>
-        </is>
-      </c>
-      <c r="D59" t="n">
-        <v>48.818819</v>
-      </c>
-      <c r="E59" t="n">
-        <v>2.319869</v>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
           <t>48.818819, 2.319869</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Pharmacie Renard</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>pharmacie</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D60" t="n">
-        <v>48.8160855</v>
-      </c>
-      <c r="E60" t="n">
-        <v>2.3085881</v>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>48.8160855, 2.3085881</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Pharmacie Tuffier</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>pharmacie</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D61" t="n">
-        <v>48.8112481</v>
-      </c>
-      <c r="E61" t="n">
-        <v>2.3145403</v>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>48.8112481, 2.3145403</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Pharmacie de Paris</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>pharmacie</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D62" t="n">
-        <v>48.8185287</v>
-      </c>
-      <c r="E62" t="n">
-        <v>2.3225912</v>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>48.8185287, 2.3225912</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Pharmacie de l'Aquapol</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>pharmacie</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D63" t="n">
-        <v>48.814625</v>
-      </c>
-      <c r="E63" t="n">
-        <v>2.32043</v>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>48.814625, 2.32043</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Pharmacie de l'Église</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>pharmacie</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D64" t="n">
-        <v>48.8178715</v>
-      </c>
-      <c r="E64" t="n">
-        <v>2.3190587</v>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>48.8178715, 2.3190587</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Pharmacie du Fort</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>pharmacie</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D65" t="n">
-        <v>48.8119254</v>
-      </c>
-      <c r="E65" t="n">
-        <v>2.3233672</v>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>48.8119254, 2.3233672</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Pharmacie du Marché</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>pharmacie</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D66" t="n">
-        <v>48.8166678</v>
-      </c>
-      <c r="E66" t="n">
-        <v>2.3212215</v>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>48.8166678, 2.3212215</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Pharmacie du Parc</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>pharmacie</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D67" t="n">
-        <v>48.8133473</v>
-      </c>
-      <c r="E67" t="n">
-        <v>2.3162607</v>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>48.8133473, 2.3162607</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Pharmacie du Square</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>pharmacie</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D68" t="n">
-        <v>48.8135808</v>
-      </c>
-      <c r="E68" t="n">
-        <v>2.3070756</v>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>48.8135808, 2.3070756</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>pharmacieCOS</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>pharmacie</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D69" t="n">
-        <v>48.8163976</v>
-      </c>
-      <c r="E69" t="n">
-        <v>2.3113604</v>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>48.8163976, 2.3113604</t>
         </is>
       </c>
     </row>

</xml_diff>